<commit_message>
Update CdaBLToBooleanConceptMap URL and comments 7745c0cf305a55fab99bb7256c8fd5ba1ff41c4e
</commit_message>
<xml_diff>
--- a/traitement-erreur/ig/CdaBLToBooleanConceptMap.xlsx
+++ b/traitement-erreur/ig/CdaBLToBooleanConceptMap.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="37">
   <si>
     <t>Property</t>
   </si>
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/DataTypes/CdaBLToFHIR</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/CdaBLToBooleanConceptMap</t>
   </si>
   <si>
     <t>Version</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-22T09:42:41+00:00</t>
+    <t>2026-07-22T12:41:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -121,6 +121,9 @@
   </si>
   <si>
     <t>boolean</t>
+  </si>
+  <si>
+    <t>Primitive Type boolean</t>
   </si>
 </sst>
 </file>
@@ -427,7 +430,7 @@
         <v>35</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>